<commit_message>
update - improved search
</commit_message>
<xml_diff>
--- a/Product_Data_File/master.xlsx
+++ b/Product_Data_File/master.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="74">
   <si>
     <t>Term Label</t>
   </si>
@@ -139,19 +139,19 @@
     <t>TC-01</t>
   </si>
   <si>
-    <t>7</t>
+    <t>7.0</t>
   </si>
   <si>
     <t>4.8</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>130</t>
-  </si>
-  <si>
-    <t>12</t>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>130.0</t>
+  </si>
+  <si>
+    <t>12.0</t>
   </si>
   <si>
     <t>0.99</t>
@@ -166,10 +166,10 @@
     <t>5.5</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>155</t>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>155.0</t>
   </si>
   <si>
     <t>1.01</t>
@@ -224,9 +224,6 @@
   </si>
   <si>
     <t>INCOMPLETE</t>
-  </si>
-  <si>
-    <t>1.004</t>
   </si>
   <si>
     <t>1.0040</t>
@@ -714,7 +711,7 @@
         <v>58</v>
       </c>
       <c r="G8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -788,7 +785,7 @@
         <v>61</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -998,7 +995,7 @@
         <v>69</v>
       </c>
       <c r="G24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1023,10 +1020,10 @@
         <v>36</v>
       </c>
       <c r="F26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
OCR cache and exit
</commit_message>
<xml_diff>
--- a/Product_Data_File/master.xlsx
+++ b/Product_Data_File/master.xlsx
@@ -88,6 +88,15 @@
     <t>Power Draw Idle Source</t>
   </si>
   <si>
+    <t>Thermal Margin Low</t>
+  </si>
+  <si>
+    <t>Thermal Soak High Status</t>
+  </si>
+  <si>
+    <t>Thermal Soak High Duration</t>
+  </si>
+  <si>
     <t>Random Vib Z Amplitude</t>
   </si>
   <si>
@@ -97,21 +106,12 @@
     <t>LVDT-2 Status</t>
   </si>
   <si>
+    <t>LVDT-2 Pre-Trim</t>
+  </si>
+  <si>
     <t>LVDT-2 Post-Trim</t>
   </si>
   <si>
-    <t>Thermal Soak High Status</t>
-  </si>
-  <si>
-    <t>Thermal Soak High Duration</t>
-  </si>
-  <si>
-    <t>Thermal Margin Low</t>
-  </si>
-  <si>
-    <t>LVDT-2 Pre-Trim</t>
-  </si>
-  <si>
     <t>Document Profile</t>
   </si>
   <si>
@@ -217,6 +217,9 @@
     <t>Table 4</t>
   </si>
   <si>
+    <t>1.5</t>
+  </si>
+  <si>
     <t>0.9989</t>
   </si>
   <si>
@@ -224,9 +227,6 @@
   </si>
   <si>
     <t>1.0040</t>
-  </si>
-  <si>
-    <t>1.5</t>
   </si>
   <si>
     <t>IData Packages/Hyperion_SV3_SN42_RevE</t>
@@ -901,22 +901,13 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
-      </c>
-      <c r="C19" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="F19" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -924,22 +915,13 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-      <c r="D20" t="s">
-        <v>46</v>
-      </c>
-      <c r="E20" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="F20" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -947,13 +929,13 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -961,13 +943,22 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" t="s">
+        <v>45</v>
+      </c>
+      <c r="E22" t="s">
+        <v>45</v>
       </c>
       <c r="F22" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="G22" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -975,13 +966,22 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="C23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" t="s">
+        <v>52</v>
       </c>
       <c r="F23" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="G23" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -989,13 +989,13 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G24" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1003,13 +1003,13 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F25" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="G25" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1020,10 +1020,10 @@
         <v>36</v>
       </c>
       <c r="F26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
patched selection and master gen
</commit_message>
<xml_diff>
--- a/Product_Data_File/master.xlsx
+++ b/Product_Data_File/master.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="62">
   <si>
     <t>Term Label</t>
   </si>
@@ -46,87 +46,84 @@
     <t>Data</t>
   </si>
   <si>
+    <t>Chamber Pressure Over</t>
+  </si>
+  <si>
+    <t>Chamber Pressure Units</t>
+  </si>
+  <si>
+    <t>Harness Resistance</t>
+  </si>
+  <si>
+    <t>Harness Resistance Quality</t>
+  </si>
+  <si>
+    <t>LVDT-2 Post-Trim</t>
+  </si>
+  <si>
+    <t>LVDT-2 Pre-Trim</t>
+  </si>
+  <si>
+    <t>LVDT-2 Status</t>
+  </si>
+  <si>
+    <t>Power Draw Idle Source</t>
+  </si>
+  <si>
+    <t>Power Draw Peak</t>
+  </si>
+  <si>
+    <t>Power Draw Peak Source</t>
+  </si>
+  <si>
     <t>Program Name</t>
   </si>
   <si>
+    <t>Random Vib Z Amplitude</t>
+  </si>
+  <si>
     <t>Serial Number</t>
   </si>
   <si>
-    <t>Date Compiled</t>
-  </si>
-  <si>
     <t>Source Bundle Path</t>
   </si>
   <si>
-    <t>Chamber Pressure Over</t>
-  </si>
-  <si>
-    <t>Chamber Pressure Units</t>
-  </si>
-  <si>
-    <t>Harness Resistance</t>
-  </si>
-  <si>
-    <t>Harness Resistance Quality</t>
+    <t>TC-02 Post Trim</t>
+  </si>
+  <si>
+    <t>Thermal Margin Low</t>
+  </si>
+  <si>
+    <t>Thermal Soak High Duration</t>
+  </si>
+  <si>
+    <t>Thermal Soak High Status</t>
+  </si>
+  <si>
+    <t>Thrust Nominal Confidence</t>
+  </si>
+  <si>
+    <t>Thrust Nominal Target</t>
   </si>
   <si>
     <t>Thrust Nominal Value</t>
   </si>
   <si>
-    <t>Thrust Nominal Target</t>
-  </si>
-  <si>
-    <t>Thrust Nominal Confidence</t>
-  </si>
-  <si>
-    <t>Power Draw Peak</t>
-  </si>
-  <si>
-    <t>Power Draw Peak Source</t>
-  </si>
-  <si>
-    <t>Power Draw Idle Source</t>
-  </si>
-  <si>
-    <t>Thermal Margin Low</t>
-  </si>
-  <si>
-    <t>Thermal Soak High Status</t>
-  </si>
-  <si>
-    <t>Thermal Soak High Duration</t>
-  </si>
-  <si>
-    <t>Random Vib Z Amplitude</t>
-  </si>
-  <si>
-    <t>TC-02 Post Trim</t>
-  </si>
-  <si>
-    <t>LVDT-2 Status</t>
-  </si>
-  <si>
-    <t>LVDT-2 Pre-Trim</t>
-  </si>
-  <si>
-    <t>LVDT-2 Post-Trim</t>
+    <t>Functional Acceptance</t>
+  </si>
+  <si>
+    <t>Calibration</t>
+  </si>
+  <si>
+    <t>Performance KPI</t>
   </si>
   <si>
     <t>Document Profile</t>
   </si>
   <si>
-    <t>Functional Acceptance</t>
-  </si>
-  <si>
-    <t>Performance KPI</t>
-  </si>
-  <si>
     <t>Environmental</t>
   </si>
   <si>
-    <t>Calibration</t>
-  </si>
-  <si>
     <t>psia</t>
   </si>
   <si>
@@ -139,103 +136,70 @@
     <t>TC-01</t>
   </si>
   <si>
-    <t>7.0</t>
-  </si>
-  <si>
-    <t>4.8</t>
-  </si>
-  <si>
-    <t>0.0</t>
-  </si>
-  <si>
-    <t>130.0</t>
+    <t>FakeProgram</t>
+  </si>
+  <si>
+    <t>SV1</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>6.1 (range violation)</t>
+  </si>
+  <si>
+    <t>resistance</t>
+  </si>
+  <si>
+    <t>1.0040</t>
+  </si>
+  <si>
+    <t>INCOMPLETE</t>
+  </si>
+  <si>
+    <t>Table 4</t>
+  </si>
+  <si>
+    <t>131</t>
+  </si>
+  <si>
+    <t>Hyperion Dragonfly Propulsion Demo</t>
   </si>
   <si>
     <t>12.0</t>
   </si>
   <si>
-    <t>0.99</t>
-  </si>
-  <si>
-    <t>8.1</t>
-  </si>
-  <si>
-    <t>5.3</t>
-  </si>
-  <si>
-    <t>5.5</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>155.0</t>
-  </si>
-  <si>
-    <t>1.01</t>
-  </si>
-  <si>
-    <t>FakeProgram</t>
-  </si>
-  <si>
-    <t>SV1</t>
-  </si>
-  <si>
-    <t>Hyperion Dragonfly Propulsion Demo</t>
-  </si>
-  <si>
     <t>SN42-AX</t>
   </si>
   <si>
-    <t>2025-01-17</t>
-  </si>
-  <si>
     <t>/Data Packages/Hyperion_SV3_SN42_RevE</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>6.1 (range violation)</t>
-  </si>
-  <si>
-    <t>resistance</t>
+    <t>0.9989</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>ERROR: Smart snap: no matching row/value</t>
+  </si>
+  <si>
+    <t>0.97</t>
   </si>
   <si>
     <t>5.32</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>0.97</t>
-  </si>
-  <si>
-    <t>131</t>
-  </si>
-  <si>
-    <t>Table 4</t>
-  </si>
-  <si>
-    <t>1.5</t>
-  </si>
-  <si>
-    <t>0.9989</t>
-  </si>
-  <si>
-    <t>INCOMPLETE</t>
-  </si>
-  <si>
-    <t>1.0040</t>
+    <t>ERROR: Smart snap: numeric values found but all out of specified range</t>
+  </si>
+  <si>
+    <t>failure</t>
+  </si>
+  <si>
+    <t>Missing</t>
   </si>
   <si>
     <t>IData Packages/Hyperion_SV3_SN42_RevE</t>
-  </si>
-  <si>
-    <t>failure</t>
-  </si>
-  <si>
-    <t>Missing</t>
   </si>
 </sst>
 </file>
@@ -593,13 +557,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
     <col min="3" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="7" width="39.7109375" customWidth="1"/>
+    <col min="6" max="6" width="42.7109375" customWidth="1"/>
+    <col min="7" max="7" width="60.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -630,10 +595,10 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="G2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -641,10 +606,10 @@
         <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="G3" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -663,13 +628,16 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -677,13 +645,13 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -691,13 +659,16 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="G7" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -705,13 +676,13 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="G8" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -719,22 +690,13 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -742,13 +704,13 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -756,19 +718,10 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" t="s">
-        <v>42</v>
-      </c>
-      <c r="E11" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
         <v>60</v>
@@ -782,10 +735,10 @@
         <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -793,19 +746,13 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" t="s">
-        <v>42</v>
-      </c>
-      <c r="E13" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="G13" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -813,19 +760,13 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" t="s">
-        <v>42</v>
-      </c>
-      <c r="E14" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="F14" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="G14" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -835,17 +776,11 @@
       <c r="B15" t="s">
         <v>34</v>
       </c>
-      <c r="D15" t="s">
-        <v>43</v>
-      </c>
-      <c r="E15" t="s">
-        <v>50</v>
-      </c>
       <c r="F15" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -853,19 +788,16 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" t="s">
-        <v>51</v>
+        <v>35</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
       </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G16" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -876,10 +808,10 @@
         <v>34</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="G17" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -890,10 +822,10 @@
         <v>34</v>
       </c>
       <c r="F18" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="G18" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -901,13 +833,16 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>34</v>
+        <v>32</v>
+      </c>
+      <c r="C19" t="s">
+        <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="G19" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -915,27 +850,24 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="G20" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>26</v>
       </c>
-      <c r="B21" t="s">
-        <v>35</v>
-      </c>
       <c r="F21" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="G21" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -945,20 +877,11 @@
       <c r="B22" t="s">
         <v>35</v>
       </c>
-      <c r="C22" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" t="s">
-        <v>45</v>
-      </c>
       <c r="F22" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="G22" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -966,22 +889,13 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
-      </c>
-      <c r="C23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" t="s">
-        <v>46</v>
-      </c>
-      <c r="E23" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="F23" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="G23" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -989,13 +903,13 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F24" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1003,27 +917,13 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" t="s">
-        <v>70</v>
-      </c>
-      <c r="G26" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>